<commit_message>
Website update 2026-06-20 17:28:22
</commit_message>
<xml_diff>
--- a/source/lasvillasweb.xlsx
+++ b/source/lasvillasweb.xlsx
@@ -8,17 +8,18 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\lasvillasdebayamon\web\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D85FF01-1933-46A5-8EE9-150CBF5A590D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F965EE9B-7228-4630-8B70-E5EAC5BDE8DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Homepage" sheetId="1" r:id="rId1"/>
-    <sheet name="Documentos" sheetId="2" r:id="rId2"/>
-    <sheet name="Números útiles" sheetId="7" r:id="rId3"/>
-    <sheet name="Enlaces útiles" sheetId="8" r:id="rId4"/>
-    <sheet name="#header" sheetId="5" r:id="rId5"/>
-    <sheet name="#footer" sheetId="6" r:id="rId6"/>
+    <sheet name="Anuncios" sheetId="9" r:id="rId2"/>
+    <sheet name="Documentos" sheetId="2" r:id="rId3"/>
+    <sheet name="Números útiles" sheetId="7" r:id="rId4"/>
+    <sheet name="Enlaces útiles" sheetId="8" r:id="rId5"/>
+    <sheet name="#header" sheetId="5" r:id="rId6"/>
+    <sheet name="#footer" sheetId="6" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="Desc">'#header'!$A$4</definedName>
@@ -46,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
   <si>
     <t>Ultima actualizacion:</t>
   </si>
@@ -111,6 +112,9 @@
   </si>
   <si>
     <t>Cada miércoles a las 7:00 p. m. se celebra una reunión informal de residentes en el gazebo. Es una oportunidad para conversar sobre asuntos de interés para la comunidad. Todos los residentes son bienvenidos.</t>
+  </si>
+  <si>
+    <t>anu</t>
   </si>
 </sst>
 </file>
@@ -642,6 +646,21 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7A94208C-A5E1-410D-86D3-F1B3F1798E0F}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{13BC1153-3F6C-40E1-89DB-D14060C3AC9B}">
   <sheetPr codeName="Foglio2"/>
   <dimension ref="A2:A5"/>
@@ -674,7 +693,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36F7898C-6129-4D6F-BF35-20B4A0C8CE7F}">
   <sheetPr codeName="Foglio3"/>
   <dimension ref="A2:A14"/>
@@ -746,7 +765,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36B8FD88-522D-4664-8FE8-C1F0587B8124}">
   <sheetPr codeName="Foglio4"/>
   <dimension ref="A2:B5"/>
@@ -782,7 +801,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9EC846B1-29CA-4378-91FD-BEA3AC8F6F48}">
   <sheetPr codeName="Foglio5"/>
   <dimension ref="A4:B6"/>
@@ -801,7 +820,7 @@
     <row r="5" spans="1:2" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A5" s="13">
         <f ca="1">NOW()</f>
-        <v>46191.512985879628</v>
+        <v>46193.724751620372</v>
       </c>
       <c r="B5" s="13"/>
     </row>
@@ -819,7 +838,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{87CF910D-75B6-4C6D-9502-D7BB38A72D1D}">
   <sheetPr codeName="Foglio6"/>
   <dimension ref="A3"/>

</xml_diff>